<commit_message>
Results: Add accessibility panel in results section
Fix: #79
- Added an Accessibility Panel component to allow users to select locations, travel times, and modes of transport.
- Updated English and French localization files with new accessibility-related strings.
- Improved styles for the accessibility panel to ensure proper positioning and visibility above the map.
</commit_message>
<xml_diff>
--- a/localisation/references/questionnaireLocalisation.xlsx
+++ b/localisation/references/questionnaireLocalisation.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Widgets" sheetId="1" state="visible" r:id="rId3"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="669" uniqueCount="438">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="709" uniqueCount="464">
   <si>
     <t xml:space="preserve">questionName</t>
   </si>
@@ -1380,6 +1380,84 @@
   <si>
     <t xml:space="preserve">Transit</t>
   </si>
+  <si>
+    <t xml:space="preserve">accessibilityPanel.title</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accessibilité</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accessibility</t>
+  </si>
+  <si>
+    <t xml:space="preserve">accessibilityPanel.locationsTitle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Locations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">accessibilityPanel.bothAddresses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Les deux</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Both</t>
+  </si>
+  <si>
+    <t xml:space="preserve">accessibilityPanel.firstAddressOnly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Logement #1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">House #1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">accessibilityPanel.secondAddressOnly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Logement #2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">House #2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">accessibilityPanel.travelTimeTitle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Temps de trajet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Travel time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">accessibilityPanel.15min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15 min.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">accessibilityPanel.30min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30 min.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">accessibilityPanel.45min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">45 min.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">accessibilityPanel.modeOfTransportTitle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mode de transport</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mode of transport</t>
+  </si>
 </sst>
 </file>
 
@@ -1391,7 +1469,7 @@
     <numFmt numFmtId="166" formatCode="General"/>
     <numFmt numFmtId="167" formatCode="@"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1534,6 +1612,12 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -1625,7 +1709,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="59">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1855,6 +1939,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -6665,6 +6753,146 @@
         <v>437</v>
       </c>
     </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>439</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>441</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>391</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>444</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>446</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>447</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>449</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B39" s="58" t="s">
+        <v>452</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>453</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B40" s="58" t="s">
+        <v>455</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B41" s="58" t="s">
+        <v>457</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B42" s="58" t="s">
+        <v>459</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>460</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B43" s="58" t="s">
+        <v>461</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>462</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>463</v>
+      </c>
+    </row>
     <row r="1048377" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1048378" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1048379" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
Results: Enhance results template with transit total time
Fix: #126
- Introduced a new TotalTimeItem component to display formatted travel time in the results section.
- Refactored time formatting logic to handle various time durations.
</commit_message>
<xml_diff>
--- a/localisation/references/questionnaireLocalisation.xlsx
+++ b/localisation/references/questionnaireLocalisation.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="789" uniqueCount="527">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="825" uniqueCount="550">
   <si>
     <t xml:space="preserve">questionName</t>
   </si>
@@ -1291,6 +1291,15 @@
     <t xml:space="preserve">Total</t>
   </si>
   <si>
+    <t xml:space="preserve">locationComparison.timeTotal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Temps de transport en commun vers les destinations fréquentes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Public transport time to frequent destinations</t>
+  </si>
+  <si>
     <t xml:space="preserve">locationComparison.costsPercentageOfIncome</t>
   </si>
   <si>
@@ -1628,6 +1637,66 @@
   </si>
   <si>
     <t xml:space="preserve">Expand the panel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">timeFormat.lessThanOneMin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt; 1 min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">timeFormat.minutes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{{count}} min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">timeFormat.hours</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{{hours}} h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">timeFormat.hoursMinutes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{{hours}} h {{minutes}} min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">timeFormat.oneDay</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 jour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">timeFormat.days</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{{count}} jours</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{{count}} days</t>
+  </si>
+  <si>
+    <t xml:space="preserve">timeFormat.oneDayHours</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 jour {{hours}} h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 day {{hours}} h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">timeFormat.daysHours</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{{days}} jours {{hours}} h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{{days}} days {{hours}} h</t>
   </si>
 </sst>
 </file>
@@ -1640,7 +1709,7 @@
     <numFmt numFmtId="166" formatCode="General"/>
     <numFmt numFmtId="167" formatCode="@"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1775,6 +1844,12 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -1866,7 +1941,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="61">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2096,6 +2171,18 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -6786,10 +6873,10 @@
       <c r="B23" s="2" t="s">
         <v>414</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="C23" s="2" t="s">
         <v>415</v>
       </c>
-      <c r="D23" s="2" t="s">
+      <c r="D23" s="1" t="s">
         <v>416</v>
       </c>
     </row>
@@ -6862,31 +6949,25 @@
       <c r="D28" s="2" t="s">
         <v>431</v>
       </c>
-      <c r="E28" s="1" t="s">
-        <v>432</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>433</v>
-      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
         <v>165</v>
       </c>
       <c r="B29" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>433</v>
+      </c>
+      <c r="D29" s="2" t="s">
         <v>434</v>
       </c>
-      <c r="C29" s="1" t="s">
+      <c r="E29" s="1" t="s">
         <v>435</v>
       </c>
-      <c r="D29" s="2" t="s">
+      <c r="F29" s="1" t="s">
         <v>436</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>437</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>438</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6894,19 +6975,19 @@
         <v>165</v>
       </c>
       <c r="B30" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="D30" s="2" t="s">
         <v>439</v>
       </c>
-      <c r="C30" s="1" t="s">
+      <c r="E30" s="1" t="s">
         <v>440</v>
       </c>
-      <c r="D30" s="2" t="s">
+      <c r="F30" s="1" t="s">
         <v>441</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>442</v>
-      </c>
-      <c r="F30" s="1" t="s">
-        <v>443</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6914,19 +6995,19 @@
         <v>165</v>
       </c>
       <c r="B31" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="D31" s="2" t="s">
         <v>444</v>
       </c>
-      <c r="C31" s="1" t="s">
+      <c r="E31" s="1" t="s">
         <v>445</v>
       </c>
-      <c r="D31" s="2" t="s">
+      <c r="F31" s="1" t="s">
         <v>446</v>
-      </c>
-      <c r="E31" s="1" t="s">
-        <v>447</v>
-      </c>
-      <c r="F31" s="1" t="s">
-        <v>448</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6934,19 +7015,19 @@
         <v>165</v>
       </c>
       <c r="B32" s="2" t="s">
+        <v>447</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>448</v>
+      </c>
+      <c r="D32" s="2" t="s">
         <v>449</v>
       </c>
-      <c r="C32" s="1" t="s">
+      <c r="E32" s="1" t="s">
         <v>450</v>
       </c>
-      <c r="D32" s="2" t="s">
+      <c r="F32" s="1" t="s">
         <v>451</v>
-      </c>
-      <c r="E32" s="1" t="s">
-        <v>452</v>
-      </c>
-      <c r="F32" s="1" t="s">
-        <v>453</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6954,16 +7035,16 @@
         <v>165</v>
       </c>
       <c r="B33" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>453</v>
+      </c>
+      <c r="D33" s="2" t="s">
         <v>454</v>
       </c>
-      <c r="C33" s="1" t="s">
+      <c r="E33" s="1" t="s">
         <v>455</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="E33" s="1" t="s">
-        <v>456</v>
       </c>
       <c r="F33" s="1" t="s">
         <v>456</v>
@@ -6980,13 +7061,13 @@
         <v>458</v>
       </c>
       <c r="D34" s="2" t="s">
+        <v>458</v>
+      </c>
+      <c r="E34" s="1" t="s">
         <v>459</v>
       </c>
-      <c r="E34" s="1" t="s">
-        <v>460</v>
-      </c>
       <c r="F34" s="1" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6994,19 +7075,19 @@
         <v>165</v>
       </c>
       <c r="B35" s="2" t="s">
+        <v>460</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>461</v>
+      </c>
+      <c r="D35" s="2" t="s">
         <v>462</v>
       </c>
-      <c r="C35" s="1" t="s">
+      <c r="E35" s="1" t="s">
         <v>463</v>
       </c>
-      <c r="D35" s="2" t="s">
+      <c r="F35" s="1" t="s">
         <v>464</v>
-      </c>
-      <c r="E35" s="1" t="s">
-        <v>465</v>
-      </c>
-      <c r="F35" s="1" t="s">
-        <v>466</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7014,12 +7095,18 @@
         <v>165</v>
       </c>
       <c r="B36" s="2" t="s">
+        <v>465</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>466</v>
+      </c>
+      <c r="D36" s="2" t="s">
         <v>467</v>
       </c>
-      <c r="C36" s="1" t="s">
+      <c r="E36" s="1" t="s">
         <v>468</v>
       </c>
-      <c r="D36" s="2" t="s">
+      <c r="F36" s="1" t="s">
         <v>469</v>
       </c>
     </row>
@@ -7030,11 +7117,11 @@
       <c r="B37" s="2" t="s">
         <v>470</v>
       </c>
-      <c r="C37" s="2" t="s">
+      <c r="C37" s="1" t="s">
         <v>471</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7042,10 +7129,10 @@
         <v>165</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>474</v>
@@ -7055,20 +7142,14 @@
       <c r="A39" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="B39" s="1" t="s">
+      <c r="B39" s="2" t="s">
         <v>475</v>
       </c>
-      <c r="C39" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="D39" s="1" t="s">
+      <c r="C39" s="2" t="s">
         <v>476</v>
       </c>
-      <c r="E39" s="2" t="s">
+      <c r="D39" s="2" t="s">
         <v>477</v>
-      </c>
-      <c r="F39" s="2" t="s">
-        <v>478</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7076,12 +7157,18 @@
         <v>165</v>
       </c>
       <c r="B40" s="1" t="s">
+        <v>478</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="D40" s="1" t="s">
         <v>479</v>
       </c>
-      <c r="C40" s="1" t="s">
+      <c r="E40" s="2" t="s">
         <v>480</v>
       </c>
-      <c r="D40" s="1" t="s">
+      <c r="F40" s="2" t="s">
         <v>481</v>
       </c>
     </row>
@@ -7092,11 +7179,11 @@
       <c r="B41" s="1" t="s">
         <v>482</v>
       </c>
-      <c r="C41" s="2" t="s">
+      <c r="C41" s="1" t="s">
         <v>483</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7104,12 +7191,12 @@
         <v>165</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>484</v>
-      </c>
-      <c r="C42" s="1" t="s">
         <v>485</v>
       </c>
-      <c r="D42" s="2" t="s">
+      <c r="C42" s="2" t="s">
+        <v>486</v>
+      </c>
+      <c r="D42" s="1" t="s">
         <v>486</v>
       </c>
     </row>
@@ -7135,10 +7222,10 @@
         <v>490</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>295</v>
+        <v>491</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7146,10 +7233,10 @@
         <v>165</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>493</v>
+        <v>295</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>494</v>
@@ -7165,7 +7252,7 @@
       <c r="C46" s="1" t="s">
         <v>496</v>
       </c>
-      <c r="D46" s="1" t="s">
+      <c r="D46" s="2" t="s">
         <v>497</v>
       </c>
     </row>
@@ -7177,10 +7264,10 @@
         <v>498</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>407</v>
+        <v>499</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7188,10 +7275,10 @@
         <v>165</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>501</v>
+        <v>407</v>
       </c>
       <c r="D48" s="1" t="s">
         <v>502</v>
@@ -7250,7 +7337,7 @@
         <v>513</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7258,13 +7345,13 @@
         <v>165</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7272,13 +7359,13 @@
         <v>165</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7286,10 +7373,10 @@
         <v>165</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="D55" s="1" t="s">
         <v>520</v>
@@ -7323,7 +7410,132 @@
         <v>526</v>
       </c>
     </row>
-    <row r="1048389" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>528</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B59" s="58" t="s">
+        <v>530</v>
+      </c>
+      <c r="C59" s="58" t="s">
+        <v>531</v>
+      </c>
+      <c r="D59" s="58" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B60" s="59" t="s">
+        <v>532</v>
+      </c>
+      <c r="C60" s="59" t="s">
+        <v>533</v>
+      </c>
+      <c r="D60" s="59" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B61" s="59" t="s">
+        <v>534</v>
+      </c>
+      <c r="C61" s="59" t="s">
+        <v>535</v>
+      </c>
+      <c r="D61" s="59" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B62" s="59" t="s">
+        <v>536</v>
+      </c>
+      <c r="C62" s="59" t="s">
+        <v>537</v>
+      </c>
+      <c r="D62" s="59" t="s">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B63" s="59" t="s">
+        <v>538</v>
+      </c>
+      <c r="C63" s="59" t="s">
+        <v>539</v>
+      </c>
+      <c r="D63" s="59" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B64" s="59" t="s">
+        <v>541</v>
+      </c>
+      <c r="C64" s="60" t="s">
+        <v>542</v>
+      </c>
+      <c r="D64" s="60" t="s">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B65" s="59" t="s">
+        <v>544</v>
+      </c>
+      <c r="C65" s="59" t="s">
+        <v>545</v>
+      </c>
+      <c r="D65" s="59" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B66" s="59" t="s">
+        <v>547</v>
+      </c>
+      <c r="C66" s="59" t="s">
+        <v>548</v>
+      </c>
+      <c r="D66" s="59" t="s">
+        <v>549</v>
+      </c>
+    </row>
     <row r="1048390" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1048391" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1048392" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
Display accessibility maps for various times
Calculate the accessibility maps for transit mode for four departure times, on the week and weekend, and add buttons in the UI to change which one to display.
Fix: #125
</commit_message>
<xml_diff>
--- a/localisation/references/questionnaireLocalisation.xlsx
+++ b/localisation/references/questionnaireLocalisation.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="825" uniqueCount="550">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="857" uniqueCount="574">
   <si>
     <t xml:space="preserve">questionName</t>
   </si>
@@ -1637,6 +1637,78 @@
   </si>
   <si>
     <t xml:space="preserve">Expand the panel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">accessibilityPanel.departureTitle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Heure de départ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Departure time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">accessibilityPanel.8am</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8 AM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">accessibilityPanel.12pm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12 PM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">accessibilityPanel.5pm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 PM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">accessibilityPanel.10pm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 PM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">accessibilityPanel.week</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Semaine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Week</t>
+  </si>
+  <si>
+    <t xml:space="preserve">accessibilityPanel.weekend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fin de semaine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weekend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">accessibilityPanel.noTransitWarningMessage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notez que l’heure de départ n’a pas d’effet pour les modes autres que le transport collectif.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Note that the departure time will have no effect for modes other than transit.</t>
   </si>
   <si>
     <t xml:space="preserve">timeFormat.lessThanOneMin</t>
@@ -1703,13 +1775,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="&quot;VRAI&quot;;&quot;VRAI&quot;;&quot;FAUX&quot;"/>
     <numFmt numFmtId="166" formatCode="General"/>
     <numFmt numFmtId="167" formatCode="@"/>
+    <numFmt numFmtId="168" formatCode="[$-C0C]General"/>
+    <numFmt numFmtId="169" formatCode="[$-C0C]@"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1844,12 +1918,6 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -1941,7 +2009,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="64">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2170,19 +2238,31 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2499,7 +2579,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="10.91"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -2576,7 +2656,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" s="14" customFormat="true" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" s="14" customFormat="true" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
         <v>25</v>
       </c>
@@ -2646,7 +2726,7 @@
       <c r="XFC2" s="15"/>
       <c r="XFD2" s="15"/>
     </row>
-    <row r="3" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="16" t="s">
         <v>30</v>
       </c>
@@ -2697,7 +2777,7 @@
       <c r="Y3" s="18"/>
       <c r="XFD3" s="19"/>
     </row>
-    <row r="4" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="176.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="16" t="s">
         <v>36</v>
       </c>
@@ -2745,7 +2825,7 @@
       <c r="Y4" s="18"/>
       <c r="XFD4" s="1"/>
     </row>
-    <row r="5" s="25" customFormat="true" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" s="25" customFormat="true" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="21" t="s">
         <v>42</v>
       </c>
@@ -2816,7 +2896,7 @@
       <c r="XFC5" s="1"/>
       <c r="XFD5" s="15"/>
     </row>
-    <row r="6" s="14" customFormat="true" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" s="14" customFormat="true" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
         <v>46</v>
       </c>
@@ -2886,7 +2966,7 @@
       <c r="XFC6" s="15"/>
       <c r="XFD6" s="26"/>
     </row>
-    <row r="7" s="18" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" s="18" customFormat="true" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="27" t="s">
         <v>50</v>
       </c>
@@ -2950,7 +3030,7 @@
       <c r="XFC7" s="1"/>
       <c r="XFD7" s="1"/>
     </row>
-    <row r="8" s="18" customFormat="true" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" s="18" customFormat="true" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="29" t="s">
         <v>52</v>
       </c>
@@ -3028,7 +3108,7 @@
       <c r="XFC8" s="1"/>
       <c r="XFD8" s="1"/>
     </row>
-    <row r="9" s="18" customFormat="true" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" s="18" customFormat="true" ht="128.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="29" t="s">
         <v>60</v>
       </c>
@@ -3175,7 +3255,7 @@
       <c r="XFC10" s="1"/>
       <c r="XFD10" s="1"/>
     </row>
-    <row r="11" s="14" customFormat="true" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" s="14" customFormat="true" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
         <v>68</v>
       </c>
@@ -3309,7 +3389,7 @@
       <c r="XFC12" s="1"/>
       <c r="XFD12" s="1"/>
     </row>
-    <row r="13" s="18" customFormat="true" ht="137.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" s="18" customFormat="true" ht="204.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="27" t="s">
         <v>73</v>
       </c>
@@ -3383,7 +3463,7 @@
       <c r="XFC13" s="1"/>
       <c r="XFD13" s="1"/>
     </row>
-    <row r="14" s="18" customFormat="true" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" s="18" customFormat="true" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="29" t="s">
         <v>79</v>
       </c>
@@ -3457,7 +3537,7 @@
       <c r="XFC14" s="1"/>
       <c r="XFD14" s="1"/>
     </row>
-    <row r="15" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
         <v>84</v>
       </c>
@@ -3492,7 +3572,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
         <v>89</v>
       </c>
@@ -3524,7 +3604,7 @@
       </c>
       <c r="XFD16" s="1"/>
     </row>
-    <row r="17" s="14" customFormat="true" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" s="14" customFormat="true" ht="176.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
         <v>91</v>
       </c>
@@ -3594,7 +3674,7 @@
       <c r="XFC17" s="15"/>
       <c r="XFD17" s="1"/>
     </row>
-    <row r="18" s="26" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" s="26" customFormat="true" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="37" t="s">
         <v>95</v>
       </c>
@@ -3768,7 +3848,7 @@
       <c r="XFC20" s="1"/>
       <c r="XFD20" s="1"/>
     </row>
-    <row r="21" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="16" t="s">
         <v>105</v>
       </c>
@@ -3817,7 +3897,7 @@
       <c r="X21" s="16"/>
       <c r="Y21" s="18"/>
     </row>
-    <row r="22" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="41" t="s">
         <v>110</v>
       </c>
@@ -3852,7 +3932,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="41" t="s">
         <v>115</v>
       </c>
@@ -3924,7 +4004,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="41" t="s">
         <v>125</v>
       </c>
@@ -3965,7 +4045,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="41" t="s">
         <v>131</v>
       </c>
@@ -4009,7 +4089,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="41" t="s">
         <v>137</v>
       </c>
@@ -4045,7 +4125,7 @@
       </c>
       <c r="XFD27" s="1"/>
     </row>
-    <row r="28" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
         <v>141</v>
       </c>
@@ -4080,7 +4160,7 @@
       </c>
       <c r="XFD28" s="1"/>
     </row>
-    <row r="29" s="25" customFormat="true" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" s="25" customFormat="true" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="21" t="s">
         <v>146</v>
       </c>
@@ -4151,7 +4231,7 @@
       <c r="XFC29" s="1"/>
       <c r="XFD29" s="1"/>
     </row>
-    <row r="30" s="14" customFormat="true" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" s="14" customFormat="true" ht="243.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
         <v>147</v>
       </c>
@@ -4390,7 +4470,7 @@
       <c r="XFC33" s="1"/>
       <c r="XFD33" s="1"/>
     </row>
-    <row r="34" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
         <v>158</v>
       </c>
@@ -4426,7 +4506,7 @@
       </c>
       <c r="XFD34" s="1"/>
     </row>
-    <row r="35" s="25" customFormat="true" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" s="25" customFormat="true" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="21" t="s">
         <v>163</v>
       </c>
@@ -4603,7 +4683,7 @@
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="7" style="34" width="8.59"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="45" t="s">
         <v>171</v>
       </c>
@@ -6222,7 +6302,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="24.39"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="54" t="s">
         <v>315</v>
       </c>
@@ -6544,7 +6624,8 @@
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16.72"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="33.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="41.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="57" width="33.83"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="19.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="19.77"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="18.91"/>
@@ -6557,7 +6638,7 @@
       <c r="B1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="58" t="s">
         <v>6</v>
       </c>
       <c r="D1" s="4" t="s">
@@ -6577,7 +6658,7 @@
       <c r="B2" s="1" t="s">
         <v>357</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="58" t="s">
         <v>358</v>
       </c>
       <c r="D2" s="4" t="s">
@@ -6593,7 +6674,7 @@
       <c r="B3" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="58" t="s">
         <v>361</v>
       </c>
       <c r="D3" s="4" t="s">
@@ -6607,7 +6688,7 @@
       <c r="B4" s="1" t="s">
         <v>363</v>
       </c>
-      <c r="C4" s="34" t="s">
+      <c r="C4" s="59" t="s">
         <v>364</v>
       </c>
       <c r="D4" s="34" t="s">
@@ -6621,7 +6702,7 @@
       <c r="B5" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="58" t="s">
         <v>366</v>
       </c>
       <c r="D5" s="4" t="s">
@@ -6635,7 +6716,7 @@
       <c r="B6" s="1" t="s">
         <v>363</v>
       </c>
-      <c r="C6" s="34" t="s">
+      <c r="C6" s="59" t="s">
         <v>368</v>
       </c>
       <c r="D6" s="34" t="s">
@@ -6649,21 +6730,21 @@
       <c r="B7" s="1" t="s">
         <v>370</v>
       </c>
-      <c r="C7" s="34" t="s">
+      <c r="C7" s="59" t="s">
         <v>371</v>
       </c>
       <c r="D7" s="34" t="s">
         <v>372</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
         <v>148</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="58" t="s">
         <v>373</v>
       </c>
       <c r="D8" s="4" t="s">
@@ -6677,7 +6758,7 @@
       <c r="B9" s="1" t="s">
         <v>363</v>
       </c>
-      <c r="C9" s="34" t="s">
+      <c r="C9" s="59" t="s">
         <v>375</v>
       </c>
       <c r="D9" s="34" t="s">
@@ -6688,10 +6769,10 @@
       <c r="A10" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="B10" s="57" t="s">
+      <c r="B10" s="60" t="s">
         <v>377</v>
       </c>
-      <c r="C10" s="34" t="s">
+      <c r="C10" s="59" t="s">
         <v>378</v>
       </c>
       <c r="D10" s="34" t="s">
@@ -6705,7 +6786,7 @@
       <c r="B11" s="1" t="s">
         <v>379</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" s="57" t="s">
         <v>380</v>
       </c>
       <c r="D11" s="1" t="s">
@@ -6719,21 +6800,21 @@
       <c r="B12" s="1" t="s">
         <v>382</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" s="57" t="s">
         <v>383</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>384</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
         <v>165</v>
       </c>
       <c r="B13" s="34" t="s">
         <v>385</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" s="61" t="s">
         <v>386</v>
       </c>
       <c r="D13" s="2" t="s">
@@ -6747,7 +6828,7 @@
       <c r="B14" s="1" t="s">
         <v>388</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" s="57" t="s">
         <v>389</v>
       </c>
       <c r="D14" s="1" t="s">
@@ -6761,7 +6842,7 @@
       <c r="B15" s="1" t="s">
         <v>391</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C15" s="57" t="s">
         <v>392</v>
       </c>
       <c r="D15" s="2" t="s">
@@ -6775,7 +6856,7 @@
       <c r="B16" s="1" t="s">
         <v>394</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C16" s="57" t="s">
         <v>395</v>
       </c>
       <c r="D16" s="2" t="s">
@@ -6789,7 +6870,7 @@
       <c r="B17" s="1" t="s">
         <v>397</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C17" s="57" t="s">
         <v>398</v>
       </c>
       <c r="D17" s="34" t="s">
@@ -6803,7 +6884,7 @@
       <c r="B18" s="1" t="s">
         <v>400</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="C18" s="57" t="s">
         <v>401</v>
       </c>
       <c r="D18" s="1" t="s">
@@ -6817,7 +6898,7 @@
       <c r="B19" s="34" t="s">
         <v>403</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C19" s="57" t="s">
         <v>404</v>
       </c>
       <c r="D19" s="1" t="s">
@@ -6831,7 +6912,7 @@
       <c r="B20" s="2" t="s">
         <v>406</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C20" s="57" t="s">
         <v>407</v>
       </c>
       <c r="D20" s="1" t="s">
@@ -6845,7 +6926,7 @@
       <c r="B21" s="2" t="s">
         <v>409</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="C21" s="57" t="s">
         <v>410</v>
       </c>
       <c r="D21" s="1" t="s">
@@ -6859,7 +6940,7 @@
       <c r="B22" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="C22" s="57" t="s">
         <v>413</v>
       </c>
       <c r="D22" s="1" t="s">
@@ -6873,7 +6954,7 @@
       <c r="B23" s="2" t="s">
         <v>414</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="C23" s="61" t="s">
         <v>415</v>
       </c>
       <c r="D23" s="1" t="s">
@@ -6887,7 +6968,7 @@
       <c r="B24" s="2" t="s">
         <v>417</v>
       </c>
-      <c r="C24" s="1" t="s">
+      <c r="C24" s="57" t="s">
         <v>418</v>
       </c>
       <c r="D24" s="2" t="s">
@@ -6901,7 +6982,7 @@
       <c r="B25" s="2" t="s">
         <v>420</v>
       </c>
-      <c r="C25" s="1" t="s">
+      <c r="C25" s="57" t="s">
         <v>421</v>
       </c>
       <c r="D25" s="2" t="s">
@@ -6915,7 +6996,7 @@
       <c r="B26" s="2" t="s">
         <v>423</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="C26" s="57" t="s">
         <v>424</v>
       </c>
       <c r="D26" s="2" t="s">
@@ -6929,7 +7010,7 @@
       <c r="B27" s="2" t="s">
         <v>426</v>
       </c>
-      <c r="C27" s="1" t="s">
+      <c r="C27" s="57" t="s">
         <v>427</v>
       </c>
       <c r="D27" s="2" t="s">
@@ -6943,7 +7024,7 @@
       <c r="B28" s="2" t="s">
         <v>429</v>
       </c>
-      <c r="C28" s="1" t="s">
+      <c r="C28" s="57" t="s">
         <v>430</v>
       </c>
       <c r="D28" s="2" t="s">
@@ -6957,7 +7038,7 @@
       <c r="B29" s="2" t="s">
         <v>432</v>
       </c>
-      <c r="C29" s="1" t="s">
+      <c r="C29" s="57" t="s">
         <v>433</v>
       </c>
       <c r="D29" s="2" t="s">
@@ -6977,7 +7058,7 @@
       <c r="B30" s="2" t="s">
         <v>437</v>
       </c>
-      <c r="C30" s="1" t="s">
+      <c r="C30" s="57" t="s">
         <v>438</v>
       </c>
       <c r="D30" s="2" t="s">
@@ -6997,7 +7078,7 @@
       <c r="B31" s="2" t="s">
         <v>442</v>
       </c>
-      <c r="C31" s="1" t="s">
+      <c r="C31" s="57" t="s">
         <v>443</v>
       </c>
       <c r="D31" s="2" t="s">
@@ -7017,7 +7098,7 @@
       <c r="B32" s="2" t="s">
         <v>447</v>
       </c>
-      <c r="C32" s="1" t="s">
+      <c r="C32" s="57" t="s">
         <v>448</v>
       </c>
       <c r="D32" s="2" t="s">
@@ -7037,7 +7118,7 @@
       <c r="B33" s="2" t="s">
         <v>452</v>
       </c>
-      <c r="C33" s="1" t="s">
+      <c r="C33" s="57" t="s">
         <v>453</v>
       </c>
       <c r="D33" s="2" t="s">
@@ -7057,7 +7138,7 @@
       <c r="B34" s="2" t="s">
         <v>457</v>
       </c>
-      <c r="C34" s="1" t="s">
+      <c r="C34" s="57" t="s">
         <v>458</v>
       </c>
       <c r="D34" s="2" t="s">
@@ -7077,7 +7158,7 @@
       <c r="B35" s="2" t="s">
         <v>460</v>
       </c>
-      <c r="C35" s="1" t="s">
+      <c r="C35" s="57" t="s">
         <v>461</v>
       </c>
       <c r="D35" s="2" t="s">
@@ -7097,7 +7178,7 @@
       <c r="B36" s="2" t="s">
         <v>465</v>
       </c>
-      <c r="C36" s="1" t="s">
+      <c r="C36" s="57" t="s">
         <v>466</v>
       </c>
       <c r="D36" s="2" t="s">
@@ -7117,7 +7198,7 @@
       <c r="B37" s="2" t="s">
         <v>470</v>
       </c>
-      <c r="C37" s="1" t="s">
+      <c r="C37" s="57" t="s">
         <v>471</v>
       </c>
       <c r="D37" s="2" t="s">
@@ -7131,7 +7212,7 @@
       <c r="B38" s="2" t="s">
         <v>473</v>
       </c>
-      <c r="C38" s="2" t="s">
+      <c r="C38" s="61" t="s">
         <v>474</v>
       </c>
       <c r="D38" s="2" t="s">
@@ -7145,7 +7226,7 @@
       <c r="B39" s="2" t="s">
         <v>475</v>
       </c>
-      <c r="C39" s="2" t="s">
+      <c r="C39" s="61" t="s">
         <v>476</v>
       </c>
       <c r="D39" s="2" t="s">
@@ -7159,7 +7240,7 @@
       <c r="B40" s="1" t="s">
         <v>478</v>
       </c>
-      <c r="C40" s="1" t="s">
+      <c r="C40" s="57" t="s">
         <v>198</v>
       </c>
       <c r="D40" s="1" t="s">
@@ -7179,7 +7260,7 @@
       <c r="B41" s="1" t="s">
         <v>482</v>
       </c>
-      <c r="C41" s="1" t="s">
+      <c r="C41" s="57" t="s">
         <v>483</v>
       </c>
       <c r="D41" s="1" t="s">
@@ -7193,7 +7274,7 @@
       <c r="B42" s="1" t="s">
         <v>485</v>
       </c>
-      <c r="C42" s="2" t="s">
+      <c r="C42" s="61" t="s">
         <v>486</v>
       </c>
       <c r="D42" s="1" t="s">
@@ -7207,7 +7288,7 @@
       <c r="B43" s="1" t="s">
         <v>487</v>
       </c>
-      <c r="C43" s="1" t="s">
+      <c r="C43" s="57" t="s">
         <v>488</v>
       </c>
       <c r="D43" s="2" t="s">
@@ -7221,7 +7302,7 @@
       <c r="B44" s="1" t="s">
         <v>490</v>
       </c>
-      <c r="C44" s="1" t="s">
+      <c r="C44" s="57" t="s">
         <v>491</v>
       </c>
       <c r="D44" s="2" t="s">
@@ -7235,7 +7316,7 @@
       <c r="B45" s="1" t="s">
         <v>493</v>
       </c>
-      <c r="C45" s="1" t="s">
+      <c r="C45" s="57" t="s">
         <v>295</v>
       </c>
       <c r="D45" s="2" t="s">
@@ -7249,7 +7330,7 @@
       <c r="B46" s="1" t="s">
         <v>495</v>
       </c>
-      <c r="C46" s="1" t="s">
+      <c r="C46" s="57" t="s">
         <v>496</v>
       </c>
       <c r="D46" s="2" t="s">
@@ -7263,7 +7344,7 @@
       <c r="B47" s="1" t="s">
         <v>498</v>
       </c>
-      <c r="C47" s="1" t="s">
+      <c r="C47" s="57" t="s">
         <v>499</v>
       </c>
       <c r="D47" s="1" t="s">
@@ -7277,7 +7358,7 @@
       <c r="B48" s="1" t="s">
         <v>501</v>
       </c>
-      <c r="C48" s="1" t="s">
+      <c r="C48" s="57" t="s">
         <v>407</v>
       </c>
       <c r="D48" s="1" t="s">
@@ -7291,7 +7372,7 @@
       <c r="B49" s="1" t="s">
         <v>503</v>
       </c>
-      <c r="C49" s="1" t="s">
+      <c r="C49" s="57" t="s">
         <v>504</v>
       </c>
       <c r="D49" s="1" t="s">
@@ -7305,7 +7386,7 @@
       <c r="B50" s="1" t="s">
         <v>506</v>
       </c>
-      <c r="C50" s="1" t="s">
+      <c r="C50" s="57" t="s">
         <v>507</v>
       </c>
       <c r="D50" s="1" t="s">
@@ -7319,7 +7400,7 @@
       <c r="B51" s="1" t="s">
         <v>509</v>
       </c>
-      <c r="C51" s="1" t="s">
+      <c r="C51" s="57" t="s">
         <v>510</v>
       </c>
       <c r="D51" s="1" t="s">
@@ -7333,7 +7414,7 @@
       <c r="B52" s="1" t="s">
         <v>512</v>
       </c>
-      <c r="C52" s="1" t="s">
+      <c r="C52" s="57" t="s">
         <v>513</v>
       </c>
       <c r="D52" s="1" t="s">
@@ -7347,7 +7428,7 @@
       <c r="B53" s="1" t="s">
         <v>515</v>
       </c>
-      <c r="C53" s="1" t="s">
+      <c r="C53" s="57" t="s">
         <v>516</v>
       </c>
       <c r="D53" s="1" t="s">
@@ -7361,7 +7442,7 @@
       <c r="B54" s="1" t="s">
         <v>517</v>
       </c>
-      <c r="C54" s="1" t="s">
+      <c r="C54" s="57" t="s">
         <v>518</v>
       </c>
       <c r="D54" s="1" t="s">
@@ -7375,7 +7456,7 @@
       <c r="B55" s="1" t="s">
         <v>519</v>
       </c>
-      <c r="C55" s="1" t="s">
+      <c r="C55" s="57" t="s">
         <v>520</v>
       </c>
       <c r="D55" s="1" t="s">
@@ -7389,7 +7470,7 @@
       <c r="B56" s="1" t="s">
         <v>521</v>
       </c>
-      <c r="C56" s="1" t="s">
+      <c r="C56" s="57" t="s">
         <v>522</v>
       </c>
       <c r="D56" s="1" t="s">
@@ -7403,7 +7484,7 @@
       <c r="B57" s="1" t="s">
         <v>524</v>
       </c>
-      <c r="C57" s="1" t="s">
+      <c r="C57" s="57" t="s">
         <v>525</v>
       </c>
       <c r="D57" s="1" t="s">
@@ -7417,133 +7498,237 @@
       <c r="B58" s="1" t="s">
         <v>527</v>
       </c>
-      <c r="C58" s="1" t="s">
+      <c r="C58" s="57" t="s">
         <v>528</v>
       </c>
       <c r="D58" s="1" t="s">
         <v>529</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="B59" s="58" t="s">
+      <c r="B59" s="1" t="s">
         <v>530</v>
       </c>
-      <c r="C59" s="58" t="s">
+      <c r="C59" s="57" t="s">
         <v>531</v>
       </c>
-      <c r="D59" s="58" t="s">
-        <v>531</v>
+      <c r="D59" s="1" t="s">
+        <v>532</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="B60" s="59" t="s">
-        <v>532</v>
-      </c>
-      <c r="C60" s="59" t="s">
+      <c r="B60" s="1" t="s">
         <v>533</v>
       </c>
-      <c r="D60" s="59" t="s">
-        <v>533</v>
+      <c r="C60" s="62" t="s">
+        <v>534</v>
+      </c>
+      <c r="D60" s="63" t="s">
+        <v>535</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="B61" s="59" t="s">
-        <v>534</v>
-      </c>
-      <c r="C61" s="59" t="s">
-        <v>535</v>
-      </c>
-      <c r="D61" s="59" t="s">
-        <v>535</v>
+      <c r="B61" s="1" t="s">
+        <v>536</v>
+      </c>
+      <c r="C61" s="62" t="s">
+        <v>537</v>
+      </c>
+      <c r="D61" s="63" t="s">
+        <v>538</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="B62" s="59" t="s">
-        <v>536</v>
-      </c>
-      <c r="C62" s="59" t="s">
-        <v>537</v>
-      </c>
-      <c r="D62" s="59" t="s">
-        <v>537</v>
+      <c r="B62" s="1" t="s">
+        <v>539</v>
+      </c>
+      <c r="C62" s="62" t="s">
+        <v>540</v>
+      </c>
+      <c r="D62" s="63" t="s">
+        <v>541</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="B63" s="59" t="s">
-        <v>538</v>
-      </c>
-      <c r="C63" s="59" t="s">
-        <v>539</v>
-      </c>
-      <c r="D63" s="59" t="s">
-        <v>540</v>
+      <c r="B63" s="1" t="s">
+        <v>542</v>
+      </c>
+      <c r="C63" s="62" t="s">
+        <v>543</v>
+      </c>
+      <c r="D63" s="63" t="s">
+        <v>544</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="B64" s="59" t="s">
-        <v>541</v>
-      </c>
-      <c r="C64" s="60" t="s">
-        <v>542</v>
-      </c>
-      <c r="D64" s="60" t="s">
-        <v>543</v>
+      <c r="B64" s="1" t="s">
+        <v>545</v>
+      </c>
+      <c r="C64" s="57" t="s">
+        <v>546</v>
+      </c>
+      <c r="D64" s="1" t="s">
+        <v>547</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="B65" s="59" t="s">
-        <v>544</v>
-      </c>
-      <c r="C65" s="59" t="s">
-        <v>545</v>
-      </c>
-      <c r="D65" s="59" t="s">
-        <v>546</v>
+      <c r="B65" s="1" t="s">
+        <v>548</v>
+      </c>
+      <c r="C65" s="57" t="s">
+        <v>549</v>
+      </c>
+      <c r="D65" s="1" t="s">
+        <v>550</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="B66" s="59" t="s">
-        <v>547</v>
-      </c>
-      <c r="C66" s="59" t="s">
-        <v>548</v>
-      </c>
-      <c r="D66" s="59" t="s">
-        <v>549</v>
-      </c>
-    </row>
-    <row r="1048390" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048391" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048392" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048393" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048394" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048395" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048396" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048397" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+      <c r="B66" s="1" t="s">
+        <v>551</v>
+      </c>
+      <c r="C66" s="61" t="s">
+        <v>552</v>
+      </c>
+      <c r="D66" s="1" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B67" s="34" t="s">
+        <v>554</v>
+      </c>
+      <c r="C67" s="59" t="s">
+        <v>555</v>
+      </c>
+      <c r="D67" s="34" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>556</v>
+      </c>
+      <c r="C68" s="61" t="s">
+        <v>557</v>
+      </c>
+      <c r="D68" s="2" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>558</v>
+      </c>
+      <c r="C69" s="61" t="s">
+        <v>559</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>560</v>
+      </c>
+      <c r="C70" s="61" t="s">
+        <v>561</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>562</v>
+      </c>
+      <c r="C71" s="61" t="s">
+        <v>563</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>565</v>
+      </c>
+      <c r="C72" s="61" t="s">
+        <v>566</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>568</v>
+      </c>
+      <c r="C73" s="61" t="s">
+        <v>569</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="C74" s="61" t="s">
+        <v>572</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>573</v>
+      </c>
+    </row>
     <row r="1048398" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1048399" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1048400" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
Add parking to utilities questions
The questions asking if the utilities are included in the rent (as well the cost of said utilities) now mention parking.
Fix: #64
</commit_message>
<xml_diff>
--- a/localisation/references/questionnaireLocalisation.xlsx
+++ b/localisation/references/questionnaireLocalisation.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Widgets" sheetId="1" state="visible" r:id="rId3"/>
@@ -394,10 +394,10 @@
     <t xml:space="preserve">areUtilitiesIncluded</t>
   </si>
   <si>
-    <t xml:space="preserve">**Le prix des services publics** (électricité, gaz, ...) **est-il inclus dans le loyer?**</t>
-  </si>
-  <si>
-    <t xml:space="preserve">**Is the cost of utilities** (electricity, gas, ...) **included in the rent?**</t>
+    <t xml:space="preserve">**Le prix des services publics** (électricité, gaz, parking, ...) **est-il inclus dans le loyer?**</t>
+  </si>
+  <si>
+    <t xml:space="preserve">**Is the cost of utilities** (electricity, gas, parking, ...) **included in the rent?**</t>
   </si>
   <si>
     <t xml:space="preserve">yesNo</t>
@@ -472,10 +472,10 @@
     <t xml:space="preserve">utilitiesMonthly</t>
   </si>
   <si>
-    <t xml:space="preserve">**Montant mensuel des services publics** (électricité, gaz, ...)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">**Monthly cost of utilities** (electricity, gas, ...)</t>
+    <t xml:space="preserve">**Montant mensuel des services publics** (électricité, gaz, parking, ...)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">**Monthly cost of utilities** (electricity, gas, parking, ...)</t>
   </si>
   <si>
     <t xml:space="preserve">askForUtilitiesCustomConditional</t>
@@ -3932,7 +3932,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="41" t="s">
         <v>115</v>
       </c>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="XFD27" s="1"/>
     </row>
-    <row r="28" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
         <v>141</v>
       </c>

</xml_diff>